<commit_message>
feat(deploy): add Vercel serverless configuration and lightweight cloud requirements
</commit_message>
<xml_diff>
--- a/Assessment2_Kevin_Johnson.xlsx
+++ b/Assessment2_Kevin_Johnson.xlsx
@@ -871,7 +871,7 @@
       </c>
       <c r="B9" s="24" t="inlineStr">
         <is>
-          <t>https://prompt-based-ai-video-editor.onrender.com/demo</t>
+          <t>https://prompt-based-ai-video-editor.vercel.app/demo</t>
         </is>
       </c>
     </row>
@@ -895,7 +895,7 @@
       </c>
       <c r="B11" s="24" t="inlineStr">
         <is>
-          <t>~45s (Render free-tier container spin-up; instant &lt; 1.0s warm)</t>
+          <t>&lt; 1.0s (Vercel Serverless Python &amp; Edge CDN; instant response)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(deploy): switch primary deployment to Render Docker container with updated Excel
</commit_message>
<xml_diff>
--- a/Assessment2_Kevin_Johnson.xlsx
+++ b/Assessment2_Kevin_Johnson.xlsx
@@ -871,7 +871,7 @@
       </c>
       <c r="B9" s="24" t="inlineStr">
         <is>
-          <t>https://prompt-based-ai-video-editor.vercel.app/demo</t>
+          <t>https://prompt-based-ai-video-editor.onrender.com/demo</t>
         </is>
       </c>
     </row>
@@ -895,7 +895,7 @@
       </c>
       <c r="B11" s="24" t="inlineStr">
         <is>
-          <t>&lt; 1.0s (Vercel Serverless Python &amp; Edge CDN; instant response)</t>
+          <t>~45s (Render free-tier container spin-up; instant &lt; 1.0s warm)</t>
         </is>
       </c>
     </row>

</xml_diff>